<commit_message>
updates for v0.2.0 odmlib
</commit_message>
<xml_diff>
--- a/define2-1-to-xlsx/data/odmlib-define-metadata.xlsx
+++ b/define2-1-to-xlsx/data/odmlib-define-metadata.xlsx
@@ -5279,24 +5279,29 @@
     <t>IE Test Codes</t>
   </si>
   <si>
-    <t>Is pregnant, nursing, or planning to become pregnant
-              within 6 months of last study treatment</t>
-  </si>
-  <si>
-    <t>Is unable or unwilling to undergo multiple
-              venipunctures</t>
-  </si>
-  <si>
-    <t>Is known to have had a substance abuse (drug or alcohol)
-              problem within the previous 3 years</t>
-  </si>
-  <si>
-    <t>Has Xyz disease of at least 10 weeks duration confirmed by
-              biopsy</t>
-  </si>
-  <si>
-    <t>Did not respond to a standard course of medication
-              Abc</t>
+    <t xml:space="preserve">Is pregnant, nursing, or planning to become pregnant
+                            within 6 months of last study treatment
+                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is unable or unwilling to undergo multiple
+                            venipunctures
+                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is known to have had a substance abuse (drug or alcohol)
+                            problem within the previous 3 years
+                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has Xyz disease of at least 10 weeks duration confirmed by
+                            biopsy
+                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Did not respond to a standard course of medication
+                            Abc
+                        </t>
   </si>
   <si>
     <t>Domain Abbreviation (LB)</t>
@@ -6601,7 +6606,9 @@
     <t>SAS 9.0 or later, as part of a data step assignment or proc sql select and update statements.</t>
   </si>
   <si>
-    <t xml:space="preserve"> catx(".",STUDYID,SUBJID) </t>
+    <t xml:space="preserve">
+                    catx(".",STUDYID,SUBJID)
+                </t>
   </si>
   <si>
     <t>Algorithm to derive VSBLFL</t>

</xml_diff>